<commit_message>
Update workflow metrics and enhance documentation for clarity
- Renamed `CountOfSteps` to `CountOfNonProposedSteps` in the schema and related files to better reflect its purpose.
- Updated formulas in the README.SCHEMA.md to align with the new naming convention.
- Added new workflow examples in the JSON files, including detailed descriptions and step counts for better understanding.
- Revised HTML and markdown reports to accurately represent the updated metrics and ensure consistency across all documentation.
- Enhanced the specification document to clarify the calculated fields and their computations, improving overall usability.
</commit_message>
<xml_diff>
--- a/execution-substrates/csv/rulebook.xlsx
+++ b/execution-substrates/csv/rulebook.xlsx
@@ -459,7 +459,7 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -506,7 +506,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>CountOfSteps</t>
+          <t>CountOfNonProposedSteps</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -518,186 +518,186 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>onboarding</t>
+          <t>performance-review</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>onboarding</t>
+          <t>performance-review</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Onboarding</t>
+          <t>Performance Review</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Employee Onboarding</t>
+          <t>Annual Performance Review</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>A step-by-step process to onboard new employees, including document collection, orientation, and training.</t>
+          <t>Structured workflow for conducting annual employee performance evaluations.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>WF-ONB-001</t>
+          <t>WF-PRV-007</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2024-05-10</t>
+          <t>2024-05-15</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>submit-request</t>
+          <t>system-notification-sent, step-2, recwwXHLqxKPhj6Mt</t>
         </is>
       </c>
       <c r="I2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J2" s="3" t="b">
         <v>1</v>
-      </c>
-      <c r="J2" s="3" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>invoice-approval</t>
+          <t>change-management</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>invoice-approval</t>
+          <t>change-management</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Invoice Approval</t>
+          <t>Change Management</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Invoice Approval Workflow</t>
+          <t>Change Management Workflow</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Automated workflow for reviewing, approving, and processing vendor invoices.</t>
+          <t>Structured process for requesting, evaluating, and implementing organizational changes.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>WF-INV-002</t>
+          <t>WF-CHM-015</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2024-06-01</t>
+          <t>2024-05-27</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>manager-review</t>
+          <t>close-workflow, step1, asdf</t>
         </is>
       </c>
       <c r="I3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J3" s="3" t="b">
         <v>1</v>
-      </c>
-      <c r="J3" s="3" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>content-publishing</t>
+          <t>asset-management</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>content-publishing</t>
+          <t>asset-management</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Content Publishing</t>
+          <t>Asset Management</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Content Publishing Process</t>
+          <t>Asset Management Process</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Workflow for drafting, reviewing, and publishing content to the company website.</t>
+          <t>Process for tracking, maintaining, and auditing company assets.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>WF-CNT-003</t>
+          <t>WF-ASM-012</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2024-05-28</t>
+          <t>2024-05-18</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>automated-eligibility-check</t>
+          <t>assign-task-to-team, some-new-task</t>
         </is>
       </c>
       <c r="I4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J4" s="3" t="b">
         <v>1</v>
-      </c>
-      <c r="J4" s="3" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>leave-request</t>
+          <t>incident-reporting</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>leave-request</t>
+          <t>incident-reporting</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Leave Request</t>
+          <t>Incident Reporting</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Leave Request Workflow</t>
+          <t>Incident Reporting Process</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Process for employees to submit, review, and approve leave requests.</t>
+          <t>Steps for reporting, investigating, and resolving workplace incidents.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>WF-LRQ-004</t>
+          <t>WF-INC-014</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2024-06-05</t>
+          <t>2024-06-06</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>finance-approval</t>
+          <t>generate-report</t>
         </is>
       </c>
       <c r="I5" s="2" t="n">
@@ -710,42 +710,42 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>it-support</t>
+          <t>customer-feedback</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>it-support</t>
+          <t>customer-feedback</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>IT Support</t>
+          <t>Customer Feedback</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>IT Support Ticketing</t>
+          <t>Customer Feedback Collection</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Workflow for submitting, triaging, and resolving IT support tickets.</t>
+          <t>Workflow for collecting, analyzing, and acting on customer feedback.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>WF-ITS-005</t>
+          <t>WF-CFB-009</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2024-05-30</t>
+          <t>2024-05-25</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>document-verification</t>
+          <t>archive-request</t>
         </is>
       </c>
       <c r="I6" s="2" t="n">
@@ -758,42 +758,42 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>expense-reimbursement</t>
+          <t>project-kickoff</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>expense-reimbursement</t>
+          <t>project-kickoff</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Expense Reimbursement</t>
+          <t>Project Kickoff</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Expense Reimbursement Process</t>
+          <t>Project Kickoff Process</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Steps for employees to submit expenses and receive reimbursements after approval.</t>
+          <t>Steps to initiate a new project, including team assignment and goal setting.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>WF-EXP-006</t>
+          <t>WF-PKO-010</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>2024-06-03</t>
+          <t>2024-05-20</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>quality-assurance-review</t>
+          <t>customer-feedback-collection</t>
         </is>
       </c>
       <c r="I7" s="2" t="n">
@@ -806,42 +806,42 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>performance-review</t>
+          <t>onboarding</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>performance-review</t>
+          <t>onboarding</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Performance Review</t>
+          <t>Onboarding</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Annual Performance Review</t>
+          <t>Employee Onboarding</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Structured workflow for conducting annual employee performance evaluations.</t>
+          <t>A step-by-step process to onboard new employees, including document collection, orientation, and training.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>WF-PRV-007</t>
+          <t>WF-ONB-001</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2024-05-15</t>
+          <t>2024-05-10</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>system-notification-sent</t>
+          <t>submit-request</t>
         </is>
       </c>
       <c r="I8" s="2" t="n">
@@ -854,42 +854,42 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>procurement</t>
+          <t>content-publishing</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>procurement</t>
+          <t>content-publishing</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Procurement</t>
+          <t>Content Publishing</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Procurement Workflow</t>
+          <t>Content Publishing Process</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Process for requesting, approving, and purchasing goods or services.</t>
+          <t>Workflow for drafting, reviewing, and publishing content to the company website.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>WF-PRC-008</t>
+          <t>WF-CNT-003</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>2024-06-02</t>
+          <t>2024-05-28</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>final-approval</t>
+          <t>automated-eligibility-check</t>
         </is>
       </c>
       <c r="I9" s="2" t="n">
@@ -902,42 +902,42 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>customer-feedback</t>
+          <t>expense-reimbursement</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>customer-feedback</t>
+          <t>expense-reimbursement</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Customer Feedback</t>
+          <t>Expense Reimbursement</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Customer Feedback Collection</t>
+          <t>Expense Reimbursement Process</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Workflow for collecting, analyzing, and acting on customer feedback.</t>
+          <t>Steps for employees to submit expenses and receive reimbursements after approval.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>WF-CFB-009</t>
+          <t>WF-EXP-006</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2024-05-25</t>
+          <t>2024-06-03</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>archive-request</t>
+          <t>quality-assurance-review</t>
         </is>
       </c>
       <c r="I10" s="2" t="n">
@@ -950,42 +950,42 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>project-kickoff</t>
+          <t>procurement</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>project-kickoff</t>
+          <t>procurement</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Project Kickoff</t>
+          <t>Procurement</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Project Kickoff Process</t>
+          <t>Procurement Workflow</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Steps to initiate a new project, including team assignment and goal setting.</t>
+          <t>Process for requesting, approving, and purchasing goods or services.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>WF-PKO-010</t>
+          <t>WF-PRC-008</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>2024-05-20</t>
+          <t>2024-06-02</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>customer-feedback-collection</t>
+          <t>final-approval</t>
         </is>
       </c>
       <c r="I11" s="2" t="n">
@@ -998,42 +998,42 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>contract-review</t>
+          <t>invoice-approval</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>contract-review</t>
+          <t>invoice-approval</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Contract Review</t>
+          <t>Invoice Approval</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Contract Review Workflow</t>
+          <t>Invoice Approval Workflow</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Workflow for legal and management review of contracts before signing.</t>
+          <t>Automated workflow for reviewing, approving, and processing vendor invoices.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>WF-CTR-011</t>
+          <t>WF-INV-002</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2024-06-04</t>
+          <t>2024-06-01</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>legal-compliance-check</t>
+          <t>manager-review</t>
         </is>
       </c>
       <c r="I12" s="2" t="n">
@@ -1046,49 +1046,49 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>asset-management</t>
+          <t>contract-review</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>asset-management</t>
+          <t>contract-review</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Asset Management</t>
+          <t>Contract Review</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Asset Management Process</t>
+          <t>Contract Review Workflow</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Process for tracking, maintaining, and auditing company assets.</t>
+          <t>Workflow for legal and management review of contracts before signing.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>WF-ASM-012</t>
+          <t>WF-CTR-011</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>2024-05-18</t>
+          <t>2024-06-04</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>assign-task-to-team, some-new-task</t>
+          <t>legal-compliance-check</t>
         </is>
       </c>
       <c r="I13" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J13" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -1142,42 +1142,42 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>incident-reporting</t>
+          <t>it-support</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>incident-reporting</t>
+          <t>it-support</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Incident Reporting</t>
+          <t>IT Support</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Incident Reporting Process</t>
+          <t>IT Support Ticketing</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Steps for reporting, investigating, and resolving workplace incidents.</t>
+          <t>Workflow for submitting, triaging, and resolving IT support tickets.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>WF-INC-014</t>
+          <t>WF-ITS-005</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>2024-06-06</t>
+          <t>2024-05-30</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>generate-report</t>
+          <t>document-verification</t>
         </is>
       </c>
       <c r="I15" s="2" t="n">
@@ -1190,42 +1190,42 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>change-management</t>
+          <t>leave-request</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>change-management</t>
+          <t>leave-request</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Change Management</t>
+          <t>Leave Request</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Change Management Workflow</t>
+          <t>Leave Request Workflow</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Structured process for requesting, evaluating, and implementing organizational changes.</t>
+          <t>Process for employees to submit, review, and approve leave requests.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>WF-CHM-015</t>
+          <t>WF-LRQ-004</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2024-05-27</t>
+          <t>2024-06-05</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>close-workflow</t>
+          <t>finance-approval</t>
         </is>
       </c>
       <c r="I16" s="2" t="n">
@@ -1246,7 +1246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1396,331 +1396,311 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>automated-eligibility-check</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>automated-eligibility-check</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Automated Eligibility Check</t>
-        </is>
-      </c>
+          <t>recwwXHLqxKPhj6Mt</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>content-publishing</t>
+          <t>performance-review</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>viewer</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>it-security-gate</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>step-3</t>
-        </is>
-      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>finance-approval</t>
+          <t>automated-eligibility-check</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>finance-approval</t>
+          <t>automated-eligibility-check</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Finance Approval</t>
+          <t>Automated Eligibility Check</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>leave-request</t>
+          <t>content-publishing</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>moderator</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="G5" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>finance-approval</t>
+          <t>it-security-gate</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>step-4</t>
+          <t>step-3</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>document-verification</t>
+          <t>finance-approval</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>document-verification</t>
+          <t>finance-approval</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Document Verification</t>
+          <t>Finance Approval</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>it-support</t>
+          <t>leave-request</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>contributor</t>
+          <t>moderator</t>
         </is>
       </c>
       <c r="G6" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>compliance-check</t>
+          <t>finance-approval</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>step-5</t>
+          <t>step-4</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>quality-assurance-review</t>
+          <t>document-verification</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>quality-assurance-review</t>
+          <t>document-verification</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Quality Assurance Review</t>
+          <t>Document Verification</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>expense-reimbursement</t>
+          <t>it-support</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>manager</t>
+          <t>contributor</t>
         </is>
       </c>
       <c r="G7" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>quality-assurance</t>
+          <t>compliance-check</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>step-6</t>
+          <t>step-5</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>system-notification-sent</t>
+          <t>quality-assurance-review</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>system-notification-sent</t>
+          <t>quality-assurance-review</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>System Notification Sent</t>
+          <t>Quality Assurance Review</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>performance-review</t>
+          <t>expense-reimbursement</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>support</t>
+          <t>manager</t>
         </is>
       </c>
       <c r="G8" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>final-authorization</t>
+          <t>quality-assurance</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>step-7</t>
+          <t>step-6</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>final-approval</t>
+          <t>system-notification-sent</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>final-approval</t>
+          <t>system-notification-sent</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Final Approval</t>
+          <t>System Notification Sent</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>procurement</t>
+          <t>performance-review</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>analyst</t>
+          <t>support</t>
         </is>
       </c>
       <c r="G9" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>manager-approval</t>
+          <t>final-authorization</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>step-8</t>
+          <t>step-7</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>archive-request</t>
+          <t>final-approval</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>archive-request</t>
+          <t>final-approval</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Archive Request</t>
+          <t>Final Approval</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>customer-feedback</t>
+          <t>procurement</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>developer</t>
+          <t>analyst</t>
         </is>
       </c>
       <c r="G10" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>it-security-gate</t>
+          <t>manager-approval</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>step-9</t>
+          <t>step-8</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>customer-feedback-collection</t>
+          <t>archive-request</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>customer-feedback-collection</t>
+          <t>archive-request</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Customer Feedback Collection</t>
+          <t>Archive Request</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>project-kickoff</t>
+          <t>customer-feedback</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>tester</t>
+          <t>developer</t>
         </is>
       </c>
       <c r="G11" s="2" t="b">
@@ -1728,115 +1708,115 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>customer-confirmation</t>
+          <t>it-security-gate</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>step-10</t>
+          <t>step-9</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>legal-compliance-check</t>
+          <t>customer-feedback-collection</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>legal-compliance-check</t>
+          <t>customer-feedback-collection</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Legal Compliance Check</t>
+          <t>Customer Feedback Collection</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>contract-review</t>
+          <t>project-kickoff</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>hr</t>
+          <t>tester</t>
         </is>
       </c>
       <c r="G12" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>legal-review</t>
+          <t>customer-confirmation</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>step-11</t>
+          <t>step-10</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>assign-task-to-team</t>
+          <t>legal-compliance-check</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>assign-task-to-team</t>
+          <t>legal-compliance-check</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Assign Task to Team</t>
+          <t>Legal Compliance Check</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>asset-management</t>
+          <t>contract-review</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>finance</t>
+          <t>hr</t>
         </is>
       </c>
       <c r="G13" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>executive-sign-off</t>
+          <t>legal-review</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>step-12</t>
+          <t>step-11</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>some-new-task</t>
+          <t>assign-task-to-team</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>some-new-task</t>
+          <t>assign-task-to-team</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Some new task</t>
+          <t>Assign Task to Team</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1845,7 +1825,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -1857,34 +1837,34 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>some-new-gate</t>
+          <t>executive-sign-off</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>assign-task-to-team</t>
+          <t>step-12</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>team-lead-review</t>
+          <t>some-new-task</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>team-lead-review</t>
+          <t>some-new-task</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Team Lead Review</t>
+          <t>Some new task</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>recruitment</t>
+          <t>asset-management</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
@@ -1892,93 +1872,93 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>guest</t>
+          <t>finance</t>
         </is>
       </c>
       <c r="G15" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>legal-review</t>
+          <t>some-new-gate</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>step-13</t>
+          <t>assign-task-to-team</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>generate-report</t>
+          <t>team-lead-review</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>generate-report</t>
+          <t>team-lead-review</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Generate Report</t>
+          <t>Team Lead Review</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>incident-reporting</t>
+          <t>recruitment</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>trainer</t>
+          <t>guest</t>
         </is>
       </c>
       <c r="G16" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>finance-approval</t>
+          <t>legal-review</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>step-14</t>
+          <t>step-13</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>close-workflow</t>
+          <t>generate-report</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>close-workflow</t>
+          <t>generate-report</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Close Workflow</t>
+          <t>Generate Report</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>change-management</t>
+          <t>incident-reporting</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>owner</t>
+          <t>trainer</t>
         </is>
       </c>
       <c r="G17" s="2" t="b">
@@ -1986,14 +1966,150 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
+          <t>finance-approval</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>step-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>close-workflow</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>close-workflow</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Close Workflow</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>change-management</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
           <t>executive-sign-off</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>step-15</t>
         </is>
       </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>step1</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>step1</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>step1</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>change-management</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>asdf</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>asdf</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>asdf</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>change-management</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>step-2</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>step-2</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Step 2</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>performance-review</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2334,9 +2450,9 @@
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2352,17 +2468,17 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>WorkflowStep</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>DisplayName</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>StepNumber</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>WorkflowStep</t>
         </is>
       </c>
     </row>
@@ -2377,18 +2493,18 @@
           <t>step-1</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>submit-request</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Step-1</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="E2" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>submit-request</t>
-        </is>
       </c>
     </row>
     <row r="3">
@@ -2402,18 +2518,18 @@
           <t>step-2</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>manager-review</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Step-2</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="E3" s="2" t="n">
         <v>2</v>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>manager-review</t>
-        </is>
       </c>
     </row>
     <row r="4">
@@ -2427,18 +2543,18 @@
           <t>step-3</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>automated-eligibility-check</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Step-3</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="E4" s="2" t="n">
         <v>3</v>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>automated-eligibility-check</t>
-        </is>
       </c>
     </row>
     <row r="5">
@@ -2452,18 +2568,18 @@
           <t>step-4</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>finance-approval</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Step-4</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="E5" s="2" t="n">
         <v>4</v>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>finance-approval</t>
-        </is>
       </c>
     </row>
     <row r="6">
@@ -2477,18 +2593,18 @@
           <t>step-5</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>document-verification</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Step-5</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="E6" s="2" t="n">
         <v>5</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>document-verification</t>
-        </is>
       </c>
     </row>
     <row r="7">
@@ -2502,18 +2618,18 @@
           <t>step-6</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>quality-assurance-review</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Step-6</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="E7" s="2" t="n">
         <v>6</v>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>quality-assurance-review</t>
-        </is>
       </c>
     </row>
     <row r="8">
@@ -2527,18 +2643,18 @@
           <t>step-7</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>system-notification-sent</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Step-7</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="E8" s="2" t="n">
         <v>7</v>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>system-notification-sent</t>
-        </is>
       </c>
     </row>
     <row r="9">
@@ -2552,18 +2668,18 @@
           <t>step-8</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>final-approval</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Step-8</t>
         </is>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="E9" s="2" t="n">
         <v>8</v>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>final-approval</t>
-        </is>
       </c>
     </row>
     <row r="10">
@@ -2577,18 +2693,18 @@
           <t>step-9</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>archive-request</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Step-9</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="E10" s="2" t="n">
         <v>9</v>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>archive-request</t>
-        </is>
       </c>
     </row>
     <row r="11">
@@ -2602,18 +2718,18 @@
           <t>step-10</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>customer-feedback-collection</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Step-10</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="E11" s="2" t="n">
         <v>10</v>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>customer-feedback-collection</t>
-        </is>
       </c>
     </row>
     <row r="12">
@@ -2627,18 +2743,18 @@
           <t>step-11</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>legal-compliance-check</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Step-11</t>
         </is>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="E12" s="2" t="n">
         <v>11</v>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>legal-compliance-check</t>
-        </is>
       </c>
     </row>
     <row r="13">
@@ -2652,18 +2768,18 @@
           <t>step-12</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>assign-task-to-team</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Step-12</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="E13" s="2" t="n">
         <v>12</v>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>assign-task-to-team</t>
-        </is>
       </c>
     </row>
     <row r="14">
@@ -2677,18 +2793,18 @@
           <t>step-13</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>team-lead-review</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Step-13</t>
         </is>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="E14" s="2" t="n">
         <v>13</v>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>team-lead-review</t>
-        </is>
       </c>
     </row>
     <row r="15">
@@ -2702,18 +2818,18 @@
           <t>step-14</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>generate-report</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>Step-14</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="E15" s="2" t="n">
         <v>14</v>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>generate-report</t>
-        </is>
       </c>
     </row>
     <row r="16">
@@ -2727,18 +2843,18 @@
           <t>step-15</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>close-workflow</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>Step-15</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="E16" s="2" t="n">
         <v>15</v>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>close-workflow</t>
-        </is>
       </c>
     </row>
     <row r="17">
@@ -2752,18 +2868,18 @@
           <t>assign-task-to-team</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>some-new-task</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>Step-16</t>
         </is>
       </c>
-      <c r="D17" s="2" t="n">
+      <c r="E17" s="2" t="n">
         <v>16</v>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>some-new-task</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement admin portal with Express backend and React frontend
- Added `run-web-portal.sh` to bootstrap the admin portal and ssotme-proxy, managing server processes and auto-creating the Postgres database.
- Created the `admin-portal` directory containing essential files: `package.json`, `package-lock.json`, `server.js`, and frontend components in `web/`.
- Updated `.gitignore` to exclude portal state and proxy log files.
- Enhanced `CLAUDE.md` to document the authoritative source of the rulebook and the admin portal's functionality.
- Modified `effortless-rulebook.json` to reflect changes in project architecture and added new fields for portal integration.
- Improved overall documentation and comments for clarity and maintainability.
</commit_message>
<xml_diff>
--- a/execution-substrates/csv/rulebook.xlsx
+++ b/execution-substrates/csv/rulebook.xlsx
@@ -8,8 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERBVersions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERBCustomizations" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -496,7 +494,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -523,12 +521,13 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>jane-smith-email-com</t>
-        </is>
-      </c>
-      <c r="B2" s="3">
-        <f>SUBSTITUTE($C2, "@", "-")</f>
-        <v/>
+          <t>cust0001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>CUST0001</t>
+        </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -537,7 +536,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Bobby</t>
+          <t>Jane</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -553,12 +552,13 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>john-doe-email-com</t>
-        </is>
-      </c>
-      <c r="B3" s="3">
-        <f>SUBSTITUTE($C3, "@", "-")</f>
-        <v/>
+          <t>cust0002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>CUST0002</t>
+        </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -567,7 +567,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Jimmy</t>
+          <t>John</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -583,12 +583,13 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>emily-jones-email-com</t>
-        </is>
-      </c>
-      <c r="B4" s="3">
-        <f>SUBSTITUTE($C4, "@", "-")</f>
-        <v/>
+          <t>cust0003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>CUST0003</t>
+        </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -597,7 +598,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Mary</t>
+          <t>Emily</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -614,349 +615,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ERBVersionId</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>BaseId</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Message</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>CommitDate</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>IsPublished</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ERBCustomizationId</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>SQLCode</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>SQLTarget</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>CustomizationType</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>03a-customize-schema-sql</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>03a-customize-schema.sql</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Customize Schema</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-- ============================================================================
--- CUSTOMIZE SCHEMA - User-defined tables and schema modifications
--- ============================================================================
--- This file is for YOUR custom schema changes that should persist across
--- regeneration of the base ERB files.
---
--- USE THIS FILE FOR:
---   - Additional tables not defined in the rulebook
---   - Extra columns on existing tables (ALTER TABLE)
---   - Custom indexes for performance tuning
---   - Custom constraints or triggers
---
--- IMPORTANT:
---   - This file runs AFTER 01-drop-and-create-tables.sql
---   - The base tables already exist when this runs
---   - This file will NOT be overwritten by ERB regeneration
---
--- ============================================================================
--- Your custom schema changes go here:
-</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Postgres</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Schema</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>03b-customize-functions-sql</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>03b-customize-functions.sql</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Customize Functions</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-- ============================================================================
--- CUSTOMIZE FUNCTIONS - User-defined calculation functions
--- ============================================================================
--- This file is for YOUR custom PostgreSQL functions that should persist
--- across regeneration of the base ERB files.
---
--- IMPORTANT:
---   - This file runs AFTER 02-create-functions.sql
---   - Base ERB calc functions already exist when this runs
---   - This file will NOT be overwritten by ERB regeneration
---
--- ============================================================================
--- Your custom functions go here:
-</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Postgres</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Functions</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>03c-customize-views-sql</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>03c-customize-views.sql</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Customize Views</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-- ============================================================================
--- CUSTOMIZE VIEWS - User-defined views and view extensions
--- ============================================================================
--- This file is for YOUR custom views that should persist across
--- regeneration of the base ERB files.
---
--- IMPORTANT:
---   - This file runs AFTER 03-create-views.sql
---   - All base vw_* views already exist when this runs
---   - This file will NOT be overwritten by ERB regeneration
---
--- ============================================================================
--- Your custom views go here:
-</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Postgres</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Views</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>03d-customize-rls-sql</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>03d-customize-rls.sql</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Customize Policies (RLS)</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-- ============================================================================
--- CUSTOMIZE POLICIES - User-defined Row Level Security policies
--- ============================================================================
--- This file is for YOUR custom RLS policies that should persist across
--- regeneration of the base ERB files.
---
--- IMPORTANT:
---   - This file runs AFTER 04-create-policies.sql
---   - Base RLS policies already exist when this runs
---   - This file will NOT be overwritten by ERB regeneration
---
--- ============================================================================
--- Your custom policies go here:
-</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Postgres</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>RLS</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>03e-customize-data-sql</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>03e-customize-data.sql</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Customize Data (Seeds / Migrations)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-- ============================================================================
--- CUSTOMIZE DATA - User-defined seed data and data migrations
--- ============================================================================
--- This file is for YOUR custom seed data that should persist across
--- regeneration of the base ERB files.
---
--- IMPORTANT:
---   - This file runs AFTER 05-insert-data.sql
---   - Base seed data already exists when this runs
---   - This file will NOT be overwritten by ERB regeneration
---
--- ============================================================================
--- Your custom data inserts go here:
-</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Postgres</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Data</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor data classes and update DbContext for new structure
- Deleted obsolete data classes: AdminPortalRuntime, AppNavigation, AppPermission, BuildPipeline, CoreDataFlow, Dependency, ExecutionSubstrate, OrchestrationComponent, ProjectConfiguration, ProjectMetadata, RulebookDomain, RulebookSourceSpoke, SsotmeProxy, and TestingFramework.
- Introduced new data classes: Client, Employee, Project, Role, TypesOfProject to align with the updated architecture.
- Updated DbContext in SoAEFContext to include new DbSet properties for Client, Employee, Project, Role, and TypesOfProject, enhancing data management capabilities.
- Improved relationships and foreign key configurations in the OnModelCreating method to support the new data structure.
</commit_message>
<xml_diff>
--- a/execution-substrates/csv/rulebook.xlsx
+++ b/execution-substrates/csv/rulebook.xlsx
@@ -8,6 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERBVersions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERBCustomizations" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -494,7 +496,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Customer</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -521,13 +523,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>cust0001</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>CUST0001</t>
-        </is>
+          <t>jane-smith-email-com</t>
+        </is>
+      </c>
+      <c r="B2" s="3">
+        <f>SUBSTITUTE($C2, "@", "-")</f>
+        <v/>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -536,7 +537,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Jane</t>
+          <t>Bobby</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -552,13 +553,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>cust0002</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>CUST0002</t>
-        </is>
+          <t>john-doe-email-com</t>
+        </is>
+      </c>
+      <c r="B3" s="3">
+        <f>SUBSTITUTE($C3, "@", "-")</f>
+        <v/>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -567,7 +567,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>John</t>
+          <t>Jimmy</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -583,13 +583,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>cust0003</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>CUST0003</t>
-        </is>
+          <t>emily-jones-email-com</t>
+        </is>
+      </c>
+      <c r="B4" s="3">
+        <f>SUBSTITUTE($C4, "@", "-")</f>
+        <v/>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -598,7 +597,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Emily</t>
+          <t>Mary</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -615,4 +614,349 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ERBVersionId</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>BaseId</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Message</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>CommitDate</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>IsPublished</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ERBCustomizationId</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>SQLCode</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>SQLTarget</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>CustomizationType</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>03a-customize-schema-sql</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>03a-customize-schema.sql</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Customize Schema</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-- ============================================================================
+-- CUSTOMIZE SCHEMA - User-defined tables and schema modifications
+-- ============================================================================
+-- This file is for YOUR custom schema changes that should persist across
+-- regeneration of the base ERB files.
+--
+-- USE THIS FILE FOR:
+--   - Additional tables not defined in the rulebook
+--   - Extra columns on existing tables (ALTER TABLE)
+--   - Custom indexes for performance tuning
+--   - Custom constraints or triggers
+--
+-- IMPORTANT:
+--   - This file runs AFTER 01-drop-and-create-tables.sql
+--   - The base tables already exist when this runs
+--   - This file will NOT be overwritten by ERB regeneration
+--
+-- ============================================================================
+-- Your custom schema changes go here:
+</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Postgres</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>03b-customize-functions-sql</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>03b-customize-functions.sql</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Customize Functions</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-- ============================================================================
+-- CUSTOMIZE FUNCTIONS - User-defined calculation functions
+-- ============================================================================
+-- This file is for YOUR custom PostgreSQL functions that should persist
+-- across regeneration of the base ERB files.
+--
+-- IMPORTANT:
+--   - This file runs AFTER 02-create-functions.sql
+--   - Base ERB calc functions already exist when this runs
+--   - This file will NOT be overwritten by ERB regeneration
+--
+-- ============================================================================
+-- Your custom functions go here:
+</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Postgres</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Functions</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>03c-customize-views-sql</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>03c-customize-views.sql</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Customize Views</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-- ============================================================================
+-- CUSTOMIZE VIEWS - User-defined views and view extensions
+-- ============================================================================
+-- This file is for YOUR custom views that should persist across
+-- regeneration of the base ERB files.
+--
+-- IMPORTANT:
+--   - This file runs AFTER 03-create-views.sql
+--   - All base vw_* views already exist when this runs
+--   - This file will NOT be overwritten by ERB regeneration
+--
+-- ============================================================================
+-- Your custom views go here:
+</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Postgres</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Views</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>03d-customize-rls-sql</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>03d-customize-rls.sql</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Customize Policies (RLS)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-- ============================================================================
+-- CUSTOMIZE POLICIES - User-defined Row Level Security policies
+-- ============================================================================
+-- This file is for YOUR custom RLS policies that should persist across
+-- regeneration of the base ERB files.
+--
+-- IMPORTANT:
+--   - This file runs AFTER 04-create-policies.sql
+--   - Base RLS policies already exist when this runs
+--   - This file will NOT be overwritten by ERB regeneration
+--
+-- ============================================================================
+-- Your custom policies go here:
+</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Postgres</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>RLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>03e-customize-data-sql</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>03e-customize-data.sql</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Customize Data (Seeds / Migrations)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-- ============================================================================
+-- CUSTOMIZE DATA - User-defined seed data and data migrations
+-- ============================================================================
+-- This file is for YOUR custom seed data that should persist across
+-- regeneration of the base ERB files.
+--
+-- IMPORTANT:
+--   - This file runs AFTER 05-insert-data.sql
+--   - Base seed data already exists when this runs
+--   - This file will NOT be overwritten by ERB regeneration
+--
+-- ============================================================================
+-- Your custom data inserts go here:
+</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Postgres</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>